<commit_message>
Polished README and small tweaks in the scraper
</commit_message>
<xml_diff>
--- a/output/books-small.xlsx
+++ b/output/books-small.xlsx
@@ -510,16 +510,16 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/a-light-in-the-attic_1000/index.html</t>
+          <t>https://books.toscrape.com/catalogue/a-light-in-the-attic_1000/index.html</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/fe/72/fe72f0532301ec28892ae79a629a293c.jpg</t>
+          <t>https://books.toscrape.com/media/cache/fe/72/fe72f0532301ec28892ae79a629a293c.jpg</t>
         </is>
       </c>
       <c r="H2" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="3">
@@ -546,16 +546,16 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/tipping-the-velvet_999/index.html</t>
+          <t>https://books.toscrape.com/catalogue/tipping-the-velvet_999/index.html</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/08/e9/08e94f3731d7d6b760dfbfbc02ca5c62.jpg</t>
+          <t>https://books.toscrape.com/media/cache/08/e9/08e94f3731d7d6b760dfbfbc02ca5c62.jpg</t>
         </is>
       </c>
       <c r="H3" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="4">
@@ -582,16 +582,16 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/soumission_998/index.html</t>
+          <t>https://books.toscrape.com/catalogue/soumission_998/index.html</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/ee/cf/eecfe998905e455df12064dba399c075.jpg</t>
+          <t>https://books.toscrape.com/media/cache/ee/cf/eecfe998905e455df12064dba399c075.jpg</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="5">
@@ -618,16 +618,16 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/sharp-objects_997/index.html</t>
+          <t>https://books.toscrape.com/catalogue/sharp-objects_997/index.html</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/c0/59/c05972805aa7201171b8fc71a5b00292.jpg</t>
+          <t>https://books.toscrape.com/media/cache/c0/59/c05972805aa7201171b8fc71a5b00292.jpg</t>
         </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="6">
@@ -654,16 +654,16 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/sapiens-a-brief-history-of-humankind_996/index.html</t>
+          <t>https://books.toscrape.com/catalogue/sapiens-a-brief-history-of-humankind_996/index.html</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/ce/5f/ce5f052c65cc963cf4422be096e915c9.jpg</t>
+          <t>https://books.toscrape.com/media/cache/ce/5f/ce5f052c65cc963cf4422be096e915c9.jpg</t>
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="7">
@@ -690,16 +690,16 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/the-requiem-red_995/index.html</t>
+          <t>https://books.toscrape.com/catalogue/the-requiem-red_995/index.html</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/6b/07/6b07b77236b7c80f42bd90bf325e69f6.jpg</t>
+          <t>https://books.toscrape.com/media/cache/6b/07/6b07b77236b7c80f42bd90bf325e69f6.jpg</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="8">
@@ -726,16 +726,16 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/the-dirty-little-secrets-of-getting-your-dream-job_994/index.html</t>
+          <t>https://books.toscrape.com/catalogue/the-dirty-little-secrets-of-getting-your-dream-job_994/index.html</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/e1/1b/e11bea016d0ae1d7e2dd46fb3cb870b7.jpg</t>
+          <t>https://books.toscrape.com/media/cache/e1/1b/e11bea016d0ae1d7e2dd46fb3cb870b7.jpg</t>
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="9">
@@ -762,16 +762,16 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/the-coming-woman-a-novel-based-on-the-life-of-the-infamous-feminist-victoria-woodhull_993/index.html</t>
+          <t>https://books.toscrape.com/catalogue/the-coming-woman-a-novel-based-on-the-life-of-the-infamous-feminist-victoria-woodhull_993/index.html</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/97/36/9736132a43b8e6e3989932218ef309ed.jpg</t>
+          <t>https://books.toscrape.com/media/cache/97/36/9736132a43b8e6e3989932218ef309ed.jpg</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="10">
@@ -798,16 +798,16 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/the-boys-in-the-boat-nine-americans-and-their-epic-quest-for-gold-at-the-1936-berlin-olympics_992/index.html</t>
+          <t>https://books.toscrape.com/catalogue/the-boys-in-the-boat-nine-americans-and-their-epic-quest-for-gold-at-the-1936-berlin-olympics_992/index.html</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/d1/2d/d12d26739b5369a6b5b3024e4d08f907.jpg</t>
+          <t>https://books.toscrape.com/media/cache/d1/2d/d12d26739b5369a6b5b3024e4d08f907.jpg</t>
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="11">
@@ -834,16 +834,16 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/the-black-maria_991/index.html</t>
+          <t>https://books.toscrape.com/catalogue/the-black-maria_991/index.html</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/d1/7a/d17a3e313e52e1be5651719e4fba1d16.jpg</t>
+          <t>https://books.toscrape.com/media/cache/d1/7a/d17a3e313e52e1be5651719e4fba1d16.jpg</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="12">
@@ -870,16 +870,16 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/starving-hearts-triangular-trade-trilogy-1_990/index.html</t>
+          <t>https://books.toscrape.com/catalogue/starving-hearts-triangular-trade-trilogy-1_990/index.html</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/a0/7e/a07ed8f1c23f7b4baf7102722680bd30.jpg</t>
+          <t>https://books.toscrape.com/media/cache/a0/7e/a07ed8f1c23f7b4baf7102722680bd30.jpg</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="13">
@@ -906,16 +906,16 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/shakespeares-sonnets_989/index.html</t>
+          <t>https://books.toscrape.com/catalogue/shakespeares-sonnets_989/index.html</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/4d/7a/4d7a79a8be80a529b277ed5c4d8ba482.jpg</t>
+          <t>https://books.toscrape.com/media/cache/4d/7a/4d7a79a8be80a529b277ed5c4d8ba482.jpg</t>
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="14">
@@ -942,16 +942,16 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/set-me-free_988/index.html</t>
+          <t>https://books.toscrape.com/catalogue/set-me-free_988/index.html</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/b8/e9/b8e91bd2fc74c3954118999238abb4b8.jpg</t>
+          <t>https://books.toscrape.com/media/cache/b8/e9/b8e91bd2fc74c3954118999238abb4b8.jpg</t>
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="15">
@@ -978,16 +978,16 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/scott-pilgrims-precious-little-life-scott-pilgrim-1_987/index.html</t>
+          <t>https://books.toscrape.com/catalogue/scott-pilgrims-precious-little-life-scott-pilgrim-1_987/index.html</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/97/27/97275841c81e66d53bf9313cba06f23e.jpg</t>
+          <t>https://books.toscrape.com/media/cache/97/27/97275841c81e66d53bf9313cba06f23e.jpg</t>
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="16">
@@ -1014,16 +1014,16 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/rip-it-up-and-start-again_986/index.html</t>
+          <t>https://books.toscrape.com/catalogue/rip-it-up-and-start-again_986/index.html</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/81/7f/817f5089c0e6e62738dce2931e7323d3.jpg</t>
+          <t>https://books.toscrape.com/media/cache/81/7f/817f5089c0e6e62738dce2931e7323d3.jpg</t>
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="17">
@@ -1050,16 +1050,16 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/our-band-could-be-your-life-scenes-from-the-american-indie-underground-1981-1991_985/index.html</t>
+          <t>https://books.toscrape.com/catalogue/our-band-could-be-your-life-scenes-from-the-american-indie-underground-1981-1991_985/index.html</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/ad/96/ad96e9c9f1664cbcb0e9627b007fb6f9.jpg</t>
+          <t>https://books.toscrape.com/media/cache/ad/96/ad96e9c9f1664cbcb0e9627b007fb6f9.jpg</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="18">
@@ -1086,16 +1086,16 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/olio_984/index.html</t>
+          <t>https://books.toscrape.com/catalogue/olio_984/index.html</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/b1/0e/b10eabab1e1c811a6d47969904fd5755.jpg</t>
+          <t>https://books.toscrape.com/media/cache/b1/0e/b10eabab1e1c811a6d47969904fd5755.jpg</t>
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="19">
@@ -1122,16 +1122,16 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/mesaerion-the-best-science-fiction-stories-1800-1849_983/index.html</t>
+          <t>https://books.toscrape.com/catalogue/mesaerion-the-best-science-fiction-stories-1800-1849_983/index.html</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/e8/1f/e81f850db9b9622c65619c9f15748de7.jpg</t>
+          <t>https://books.toscrape.com/media/cache/e8/1f/e81f850db9b9622c65619c9f15748de7.jpg</t>
         </is>
       </c>
       <c r="H19" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="20">
@@ -1158,16 +1158,16 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/libertarianism-for-beginners_982/index.html</t>
+          <t>https://books.toscrape.com/catalogue/libertarianism-for-beginners_982/index.html</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/91/a4/91a46253e165d144ef5938f2d456b88f.jpg</t>
+          <t>https://books.toscrape.com/media/cache/91/a4/91a46253e165d144ef5938f2d456b88f.jpg</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
     <row r="21">
@@ -1194,16 +1194,16 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/catalogue/its-only-the-himalayas_981/index.html</t>
+          <t>https://books.toscrape.com/catalogue/its-only-the-himalayas_981/index.html</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>http://books.toscrape.com/media/cache/6d/41/6d418a73cc7d4ecfd75ca11d854041db.jpg</t>
+          <t>https://books.toscrape.com/media/cache/6d/41/6d418a73cc7d4ecfd75ca11d854041db.jpg</t>
         </is>
       </c>
       <c r="H21" s="4" t="n">
-        <v>46241.29362268518</v>
+        <v>46241.32887731482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>